<commit_message>
Infant-child form through first visit to 6 month olds
</commit_message>
<xml_diff>
--- a/forms/app/infant-child.xlsx
+++ b/forms/app/infant-child.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="4" count="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23" count="23">
   <si>
     <t>type</t>
   </si>
@@ -37,13 +37,70 @@
   </si>
   <si>
     <t>label::sw</t>
+  </si>
+  <si>
+    <t>begin group</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>child_consent</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>end group</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>calculate</t>
+  </si>
+  <si>
+    <t>consent</t>
+  </si>
+  <si>
+    <t>select_one yes_no</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>SEMA: Habari mama? Kama tulivyozungumza wakati wa matembeleo yetu yaliyopita kuwa ntakuja kukutembelea kwa ajili ya kujua maendeleo na afya ya mtoto/watoto, na pia kujadiliana na wewe pamoja na familia juu ya malezi na makuzi bora ya mtoto/watoto wako. Nafahamu kuwa unajua jinsi ya kumtunza mtoto wako na kumkuza vizuri, lakini hii ni kama nyongeza tu ya elimu kutokana na ongezeko la maradhi na matatizo mbali mbali yanayoweza kudhoofisha afya  na makuzi bora ya mtoto.</t>
+  </si>
+  <si>
+    <t>first_visit_6_months</t>
+  </si>
+  <si>
+    <t>delivery_location</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>${child_birthweight} &lt; 2 or selected(${child_size_birth},"small")</t>
+  </si>
+  <si>
+    <t>selected(${has_received_small_baby_services},"no")</t>
+  </si>
+  <si>
+    <t>yes_no</t>
+  </si>
+  <si>
+    <t>child_size</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -62,6 +119,16 @@
       <name val="Cambria"/>
       <vertAlign val="baseline"/>
       <sz val="12"/>
+      <strike val="0"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <u val="none"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <vertAlign val="baseline"/>
+      <sz val="11"/>
       <strike val="0"/>
     </font>
   </fonts>
@@ -98,10 +165,10 @@
     <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0" textRotation="0" indent="0"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0" textRotation="0" indent="0"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0" textRotation="0" indent="0"/>
     </xf>
   </cellXfs>
@@ -113,12 +180,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" style="0" width="4.856850961538462" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" style="0" width="5.999639423076924" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" style="0" width="8.71376201923077" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="0" width="11.713581730769231" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" style="0" width="13.427764423076924" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" style="0" width="54.42530048076924" customWidth="1"/>
     <col min="4" max="4" style="0" width="8.999459134615385" bestFit="1" customWidth="1"/>
     <col min="5" max="6" style="0" width="8.428064903846154" bestFit="1" customWidth="1"/>
     <col min="7" max="7" style="0" width="11.570733173076924" bestFit="1" customWidth="1"/>
@@ -126,92 +193,571 @@
     <col min="9" max="9" style="0" width="9.99939903846154" bestFit="1" customWidth="1"/>
     <col min="10" max="10" style="0" width="22.855769230769234" bestFit="1" customWidth="1"/>
     <col min="11" max="11" style="0" width="23.141466346153848" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" style="0" width="10.856490384615386" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" style="0" width="21.427283653846157" bestFit="1" customWidth="1"/>
     <col min="13" max="13" style="0" width="11.999278846153848" bestFit="1" customWidth="1"/>
     <col min="14" max="14" style="0" width="7.713822115384616" bestFit="1" customWidth="1"/>
     <col min="15" max="15" style="0" width="7.9995192307692315" bestFit="1" customWidth="1"/>
     <col min="16" max="16" style="0" width="7.285276442307693" bestFit="1" customWidth="1"/>
     <col min="17" max="17" style="0" width="12.856370192307693" bestFit="1" customWidth="1"/>
-    <col min="18" max="256" style="0" width="9.142307692307693"/>
+    <col min="18" max="16384" style="0" width="9.142307692307693"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="13.5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>read_only</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>constraint_message::en</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>constraint_message::sw</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>calculation</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>choice_filter</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>hint::en</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>hint::sw</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>repeat_count</t>
         </is>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="13.5">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="13.5">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="13.5">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>num_child_visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="13.5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>begin group </t>
+        </is>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="13.5">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>contact_id</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Contact ID of the logged in user</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="13.5">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>facility_id</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Facility ID for the parent user</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="13.5">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Name of the logged in user</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="13.5">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="13.5">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="13.5">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="13.5">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="13.5">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>date_of_birth</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="13.5">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="13.5">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>end group </t>
+        </is>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="13.5">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>child_name</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>../inputs/contact/name</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="13.5">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>n_child_visits</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>../inputs/num_child_visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="13.5">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>${n_child_visits}=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Greet the family and invite others to join the conversation as appropriate.
+SAY: I'd like to enroll ${child_name} into infant and child services.  I'll do a first check-up on their health today, and them return at important times as they grow up to make sure they are healthy and well.  Is that OK?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="13.5">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>selected(${child_consent},"yes")</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="13.5">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>child_visit_intro_note</t>
+        </is>
+      </c>
+      <c r="C21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="13.5">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>First visit to a child under 6 months old</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>${n_child_visits}=0 and ${child_consent}="yes" and (decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt; 182.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="13.5">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>select_one delivery_location</t>
+        </is>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Where was the child born?</t>
+        </is>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="13.5">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>child_card_available</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Is the child card available?</t>
+        </is>
+      </c>
+      <c r="E24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="13.5">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>birthweight_on_child_card</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Is the birthweight written on the child card?</t>
+        </is>
+      </c>
+      <c r="E25" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>selected(${child_card_available},"yes")</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="13.5">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>child_birthweight</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Enter brithweight of the child, in KG</t>
+        </is>
+      </c>
+      <c r="E26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>selected(${child_card_available},"yes") and selected(${birthweight_on_child_card},"yes")</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>. &gt;= 0.5 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Enter a number between 0.5 and 7 KG</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="13.5">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>select_one child_size</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>child_size_birth</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Approximately how large was the baby at birth?</t>
+        </is>
+      </c>
+      <c r="E27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>(selected(${birthweight_on_child_card","no") or selected(${child_card_available},"no"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="13.5">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>normal_baby_note</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>This is a normal size baby and needs normal care. You will learn about care for the normal baby in later sessions.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>${child_birthweight} &gt;= 2 or selected(${child_size_birth},"regular") or selected(${child_size_birth},"large")</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="13.5">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>small_baby_note</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>This child is a small baby and extra care and attention is needed from both CHV and family. We will talk about some of the special care your baby needs.</t>
+        </is>
+      </c>
+      <c r="F29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="13.5">
+      <c r="A30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>has_received_small_baby_services</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ASK: Have you received small baby services at the hospital?</t>
+        </is>
+      </c>
+      <c r="E30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="13.5">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>refer_small_baby_note</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>_Refer to nearest KMC ward_</t>
+        </is>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="13.5">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>encourage_small_baby_note</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>_Look child card and/or KMC booklet for next scheduled follow-up visit. Advise mother to return to the facility for scheduled follow up visits_</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>selected(${has_received_small_baby_services},"yes")</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="13.5">
+      <c r="A33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -231,30 +777,158 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" style="0" width="12.856370192307693" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="0" width="16.71328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" style="0" width="7.713822115384616" bestFit="1" customWidth="1"/>
     <col min="3" max="3" style="0" width="11.713581730769231" bestFit="1" customWidth="1"/>
     <col min="4" max="4" style="0" width="11.85643028846154" bestFit="1" customWidth="1"/>
-    <col min="5" max="256" style="0" width="9.142307692307693"/>
+    <col min="5" max="16384" style="0" width="9.142307692307693"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="14.25">
+      <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ndiyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="14.25">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Hapana</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="13.5">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>at_home</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>At home</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="13.5">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>health_facility</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>In a health facility</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="13.5">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>on_way_health_facility</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>On the way to the health facility</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="13.5">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="13.5">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="13.5">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -283,36 +957,36 @@
     <col min="4" max="4" style="0" width="6.571033653846155" bestFit="1" customWidth="1"/>
     <col min="5" max="5" style="0" width="6.428185096153847" bestFit="1" customWidth="1"/>
     <col min="6" max="6" style="0" width="19.713100961538462" bestFit="1" customWidth="1"/>
-    <col min="7" max="256" style="0" width="9.142307692307693"/>
+    <col min="7" max="16384" style="0" width="9.142307692307693"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>style</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>path</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>instance_name</t>
         </is>

</xml_diff>

<commit_message>
Most basic infant-child form and json settings to show in app
</commit_message>
<xml_diff>
--- a/forms/app/infant-child.xlsx
+++ b/forms/app/infant-child.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23" count="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24" count="24">
   <si>
     <t>type</t>
   </si>
@@ -48,9 +48,6 @@
     <t>string</t>
   </si>
   <si>
-    <t>child_consent</t>
-  </si>
-  <si>
     <t>user</t>
   </si>
   <si>
@@ -87,7 +84,13 @@
     <t>${child_birthweight} &lt; 2 or selected(${child_size_birth},"small")</t>
   </si>
   <si>
-    <t>selected(${has_received_small_baby_services},"no")</t>
+    <t>child_danger_signs</t>
+  </si>
+  <si>
+    <t>neonatal_screening</t>
+  </si>
+  <si>
+    <t>neonatal_danger_signs</t>
   </si>
   <si>
     <t>yes_no</t>
@@ -180,7 +183,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" style="0" width="11.713581730769231" bestFit="1" customWidth="1"/>
@@ -298,8 +301,10 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>child_consent</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:17" ht="13.5">
@@ -319,7 +324,7 @@
         </is>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="13.5">
@@ -367,10 +372,10 @@
     </row>
     <row r="9" spans="1:17" ht="13.5">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="13.5">
@@ -378,7 +383,7 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="13.5">
@@ -411,10 +416,10 @@
     </row>
     <row r="14" spans="1:17" ht="13.5">
       <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
         <v>9</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="13.5">
@@ -429,7 +434,7 @@
     </row>
     <row r="16" spans="1:17" ht="13.5">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -444,7 +449,7 @@
     </row>
     <row r="17" spans="1:17" ht="13.5">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -459,238 +464,232 @@
     </row>
     <row r="18" spans="1:17" ht="13.5">
       <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>previous_child_consent</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>../inputs/child_consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="13.5">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>child_date_of_birth</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>../inputs/contact/date_of_birth</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="13.5">
+      <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>${n_child_visits}=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A21" t="s">
         <v>12</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Consent</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>${n_child_visits}=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>child_consent_today</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>Greet the family and invite others to join the conversation as appropriate.
 SAY: I'd like to enroll ${child_name} into infant and child services.  I'll do a first check-up on their health today, and them return at important times as they grow up to make sure they are healthy and well.  Is that OK?</t>
         </is>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="13.5">
-      <c r="A20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>selected(${child_consent},"yes")</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="13.5">
-      <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>child_visit_intro_note</t>
-        </is>
-      </c>
-      <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
-        <v>15</v>
-      </c>
-    </row>
     <row r="22" spans="1:17" ht="13.5">
       <c r="A22" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>First visit to a child under 6 months old</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>${n_child_visits}=0 and ${child_consent}="yes" and (decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt; 182.5</t>
-        </is>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="13.5">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>select_one delivery_location</t>
-        </is>
-      </c>
-      <c r="B23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Where was the child born?</t>
-        </is>
-      </c>
-      <c r="E23" t="s">
-        <v>18</v>
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>child_visit_intro_note</t>
+        </is>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>selected(${child_consent},"yes")</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:17" ht="13.5">
       <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>First Infant Visit</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>${n_child_visits}=0 and ${child_consent}="yes" and (decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt; 182.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="13.5">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>select_one delivery_location</t>
+        </is>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Where was the child born?</t>
+        </is>
+      </c>
+      <c r="E25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="13.5">
+      <c r="A26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>child_card_available</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Is the child card available?</t>
         </is>
       </c>
-      <c r="E24" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" ht="13.5">
-      <c r="A25" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" t="inlineStr">
+      <c r="E26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="13.5">
+      <c r="A27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>birthweight_on_child_card</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Is the birthweight written on the child card?</t>
         </is>
       </c>
-      <c r="E25" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="E27" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>selected(${child_card_available},"yes")</t>
         </is>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="13.5">
-      <c r="A26" t="inlineStr">
+    <row r="28" spans="1:17" ht="13.5">
+      <c r="A28" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>child_birthweight</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Enter brithweight of the child, in KG</t>
         </is>
       </c>
-      <c r="E26" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E28" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>selected(${child_card_available},"yes") and selected(${birthweight_on_child_card},"yes")</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>. &gt;= 0.5 and . &lt;= 7</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Enter a number between 0.5 and 7 KG</t>
         </is>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="13.5">
-      <c r="A27" t="inlineStr">
+    <row r="29" spans="1:17" ht="13.5">
+      <c r="A29" t="inlineStr">
         <is>
           <t>select_one child_size</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>child_size_birth</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Approximately how large was the baby at birth?</t>
         </is>
       </c>
-      <c r="E27" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>(selected(${birthweight_on_child_card","no") or selected(${child_card_available},"no"))</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" spans="1:17" ht="13.5">
-      <c r="A28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>normal_baby_note</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>This is a normal size baby and needs normal care. You will learn about care for the normal baby in later sessions.</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>${child_birthweight} &gt;= 2 or selected(${child_size_birth},"regular") or selected(${child_size_birth},"large")</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" spans="1:17" ht="13.5">
-      <c r="A29" t="s">
-        <v>14</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>small_baby_note</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>This child is a small baby and extra care and attention is needed from both CHV and family. We will talk about some of the special care your baby needs.</t>
-        </is>
-      </c>
-      <c r="F29" t="s">
-        <v>19</v>
+      <c r="E29" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>(selected(${birthweight_on_child_card},"no") or selected(${child_card_available},"no"))</t>
+        </is>
       </c>
     </row>
     <row r="30" spans="1:17" ht="13.5">
@@ -699,65 +698,206 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>has_received_small_baby_services</t>
+          <t>normal_baby_note</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ASK: Have you received small baby services at the hospital?</t>
-        </is>
-      </c>
-      <c r="E30" t="s">
-        <v>18</v>
-      </c>
-      <c r="F30" t="s">
-        <v>19</v>
+          <t>This is a normal size baby and needs normal care. You will learn about care for the normal baby in later sessions.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>${child_birthweight} &gt;= 2 or selected(${child_size_birth},"regular") or selected(${child_size_birth},"large")</t>
+        </is>
       </c>
     </row>
     <row r="31" spans="1:17" ht="13.5">
       <c r="A31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>refer_small_baby_note</t>
+          <t>small_baby_note</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>_Refer to nearest KMC ward_</t>
+          <t>This child is a small baby and extra care and attention is needed from both CHV and family. We will talk about some of the special care your baby needs.</t>
         </is>
       </c>
       <c r="F31" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="13.5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>encourage_small_baby_note</t>
+          <t>has_received_small_baby_services</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_Look child card and/or KMC booklet for next scheduled follow-up visit. Advise mother to return to the facility for scheduled follow up visits_</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>selected(${has_received_small_baby_services},"yes")</t>
-        </is>
+          <t>ASK: Have you received small baby services at the hospital?</t>
+        </is>
+      </c>
+      <c r="E32" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="13.5">
       <c r="A33" t="s">
-        <v>9</v>
-      </c>
-      <c r="B33" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>refer_small_baby_note</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>_Refer to nearest KMC ward_</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>selected(${has_received_small_baby_services},"no")</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="13.5">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>refer_flag_small_baby</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>if(selected(${has_received_small_baby_services},"no"),1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="13.5">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>encourage_small_baby_note</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>_Look child card and/or KMC booklet for next scheduled follow-up visit. Advise mother to return to the facility for scheduled follow up visits_</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>selected(${has_received_small_baby_services},"yes")</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="13.5">
+      <c r="A36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" ht="13.5">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Child Danger Signs Screening</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>${previous_child_consent}=1 or ${child_consent_today}=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A38" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>danger_signs_intro_note</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>I'm not going to screen your chlid for danger signs.  Observe the child and discuss each danger sign with the mother and child.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="13.5">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Neonatal Danger Signs Screening</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>(decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt;= 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>select_multiple neonatal_danger_signs</t>
+        </is>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SAY: I’m now going to screen your baby for neonatal danger signs.
+Observe and discuss each danger sign with the mother and child.  Select any of the danger signs that the baby has right now</t>
+        </is>
+      </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" ht="13.5">
+      <c r="A41" t="s">
+        <v>8</v>
+      </c>
+      <c r="B41" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="13.5">
+      <c r="A42" t="s">
+        <v>8</v>
+      </c>
+      <c r="B42" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +917,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" style="0" width="16.71328125" bestFit="1" customWidth="1"/>
@@ -805,10 +945,10 @@
     </row>
     <row r="2" spans="1:4" ht="14.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -823,7 +963,7 @@
     </row>
     <row r="3" spans="1:4" ht="14.25">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -843,7 +983,7 @@
     </row>
     <row r="4" spans="1:4" ht="13.5">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -858,7 +998,7 @@
     </row>
     <row r="5" spans="1:4" ht="13.5">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -873,7 +1013,7 @@
     </row>
     <row r="6" spans="1:4" ht="13.5">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -888,7 +1028,7 @@
     </row>
     <row r="7" spans="1:4" ht="13.5">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -903,7 +1043,7 @@
     </row>
     <row r="8" spans="1:4" ht="13.5">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -918,7 +1058,7 @@
     </row>
     <row r="9" spans="1:4" ht="13.5">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -928,6 +1068,216 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="13.5">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>not_able_feed</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Not able to feed since birth, or stopped feeding well </t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="13.5">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>had_convulsions</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Had convulsions</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="13.5">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>difficulty_fast_breathing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Difficulty or fast breathing (Two counts of 60 breaths or more in one minute)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="13.5">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fever</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fever or high temperature </t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="13.5">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cold or low temperature </t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="13.5">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>yellow_pale_palms</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yellow or pale palms and soles (hands and feet), and lips. Soles should be red/pink.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="13.5">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>no_movement</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Movement only when stimulated, or no movement even on stimulation </t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="13.5">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cord_bleeding</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cord red, bleeding, or draining pus</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="13.5">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>diarrhea</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Diarrhea</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="13.5">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>eyes_pus</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Eyes draining pus</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="13.5">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>skin_boils</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Skin boils</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="13.5">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>excessive_vomiting</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Excessive vomiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="13.5">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>excessive_crying</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Excessive crying or restlessness for more than one hour, non-stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="13.5">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>None of the above</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Infant-child form through danger signs screening
</commit_message>
<xml_diff>
--- a/forms/app/infant-child.xlsx
+++ b/forms/app/infant-child.xlsx
@@ -81,16 +81,16 @@
     <t>yes</t>
   </si>
   <si>
-    <t>${child_birthweight} &lt; 2 or selected(${child_size_birth},"small")</t>
+    <t>(selected(${child_card_available},"yes") and selected(${birthweight_on_child_card},"yes") and ${child_birthweight} &lt; 2) or selected(${child_size_birth},"small")</t>
+  </si>
+  <si>
+    <t>neonatal_danger_signs</t>
+  </si>
+  <si>
+    <t>neonatal_danger_signs_secondary</t>
   </si>
   <si>
     <t>child_danger_signs</t>
-  </si>
-  <si>
-    <t>neonatal_screening</t>
-  </si>
-  <si>
-    <t>neonatal_danger_signs</t>
   </si>
   <si>
     <t>yes_no</t>
@@ -183,7 +183,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:Q119"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" style="0" width="11.713581730769231" bestFit="1" customWidth="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>selected(${child_consent},"yes")</t>
+          <t>selected(${child_consent_today},"yes")</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>${n_child_visits}=0 and ${child_consent}="yes" and (decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt; 182.5</t>
+          <t>${n_child_visits}=0 and ${child_consent_today}="yes" and (decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt; 182.5</t>
         </is>
       </c>
     </row>
@@ -823,12 +823,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Child Danger Signs Screening</t>
+          <t>Neonatal Danger Signs Screening</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>${previous_child_consent}=1 or ${child_consent_today}=1</t>
+          <t>(decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt;= 42 and (${previous_child_consent}="yes" or selected(${child_consent_today},"yes"))</t>
         </is>
       </c>
     </row>
@@ -838,46 +838,49 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>danger_signs_intro_note</t>
+          <t>neonatal_danger_signs_note</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>I'm not going to screen your chlid for danger signs.  Observe the child and discuss each danger sign with the mother and child.</t>
-        </is>
+          <t>SAY: I’m now going to screen your baby for neonatal danger signs.
+Observe and discuss each danger sign with the mother and child.  Does the baby have any of the following danger signs right now?</t>
+        </is>
+      </c>
+      <c r="E38" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:17" ht="13.5">
       <c r="A39" t="s">
-        <v>4</v>
-      </c>
-      <c r="B39" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>neonatal_not_able_feed</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Neonatal Danger Signs Screening</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>(decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt;= 42</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>select_multiple neonatal_danger_signs</t>
-        </is>
-      </c>
-      <c r="B40" t="s">
-        <v>21</v>
+          <t>Not able to feed since birth, or stopped feeding well </t>
+        </is>
+      </c>
+      <c r="E39" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" ht="13.5">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>neonatal_had_convulsions</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAY: I’m now going to screen your baby for neonatal danger signs.
-Observe and discuss each danger sign with the mother and child.  Select any of the danger signs that the baby has right now</t>
+          <t>Had convulsions</t>
         </is>
       </c>
       <c r="E40" t="s">
@@ -886,20 +889,667 @@
     </row>
     <row r="41" spans="1:17" ht="13.5">
       <c r="A41" t="s">
-        <v>8</v>
-      </c>
-      <c r="B41" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>neonatal_difficulty_fast_breathing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Difficulty or fast breathing (Two counts of 60 breaths or more in one minute)</t>
+        </is>
+      </c>
+      <c r="E41" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="13.5">
       <c r="A42" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>neonatal_fever</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Fever or high temperature </t>
+        </is>
+      </c>
+      <c r="E42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="13.5">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>neonatal_cold</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Cold or low temperature </t>
+        </is>
+      </c>
+      <c r="E43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="13.5">
+      <c r="A44" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>neonatal_yellow_pale_palms</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Yellow or pale palms and soles (hands and feet), and lips. Soles should be red/pink.</t>
+        </is>
+      </c>
+      <c r="E44" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" ht="13.5">
+      <c r="A45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>neonatal_no_movement</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Movement only when stimulated, or no movement even on stimulation </t>
+        </is>
+      </c>
+      <c r="E45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="13.5">
+      <c r="A46" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>neonatal_cord_bleeding</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Cord red, bleeding, or draining pus</t>
+        </is>
+      </c>
+      <c r="E46" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="13.5">
+      <c r="A47" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>neonatal_diarrhea</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Diarrhea</t>
+        </is>
+      </c>
+      <c r="E47" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" ht="13.5">
+      <c r="A48" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>neonatal_eyes_pus</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Eyes draining pus</t>
+        </is>
+      </c>
+      <c r="E48" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="13.5">
+      <c r="A49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>neonatal_skin_boils</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Skin boils</t>
+        </is>
+      </c>
+      <c r="E49" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="13.5">
+      <c r="A50" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>neonatal_excessive_vomiting</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Excessive vomiting</t>
+        </is>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="13.5">
+      <c r="A51" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>neonatal_excessive_crying</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Excessive crying or restlessness for more than one hour, non-stop</t>
+        </is>
+      </c>
+      <c r="E51" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" ht="13.5">
+      <c r="A52" t="s">
+        <v>10</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>refer_neonatal_danger_sign_flag</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>if(selected(${neonatal_not_able_feed},'yes') or selected(${neonatal_had_convulsions},'yes') or selected(${neonatal_difficulty_fast_breathing},'yes') or selected(${neonatal_fever},'yes') or selected(${neonatal_cold},'yes') or selected(${neonatal_yellow_pale_palms},'yes') or selected(${neonatal_no_movement},'yes') or selected(${neonatal_cord_bleeding},'yes') or selected(${neonatal_diarrhea},'yes') or selected(${neonatal_eyes_pus},'yes') or selected(${neonatal_skin_boils},'yes') or selected(${neonatal_excessive_vomiting},'yes') or selected(${neonatal_excessive_crying},'yes'),1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>has_neonatal_danger_note</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Your baby has a danger sign. This is an URGENT and super serious emergency. You should take the baby IMMEDIATELY to the nearest facility. If it is closed, you need to go to the closest hospital.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>${refer_neonatal_danger_sign_flag}=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:17" ht="13.5">
+      <c r="A54" t="s">
         <v>8</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B54" t="s">
         <v>19</v>
       </c>
     </row>
+    <row r="55" spans="1:17" ht="13.5">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Other Neonatal Danger Signs Screening</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>(decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &lt;= 42 and ${refer_neonatal_danger_sign_flag}=0 and (${previous_child_consent}="yes" or selected(${child_consent_today},"yes"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="13.5">
+      <c r="A56" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>neonatal_not_crying</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Not crying</t>
+        </is>
+      </c>
+      <c r="E56" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" ht="13.5">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>neonatal_blue_color</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Blue in color</t>
+        </is>
+      </c>
+      <c r="E57" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" ht="13.5">
+      <c r="A58" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>neonatal_eye_discharge</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Eye discharge or swollen eyes</t>
+        </is>
+      </c>
+      <c r="E58" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" ht="13.5">
+      <c r="A59" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>neonatal_skin_rash</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Skin rash</t>
+        </is>
+      </c>
+      <c r="E59" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" ht="13.5">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>neonatal_congenital</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Congenital abnormality</t>
+        </is>
+      </c>
+      <c r="E60" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" ht="13.5">
+      <c r="A61" t="s">
+        <v>12</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>neonatal_vomiting</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Occasional vomiting</t>
+        </is>
+      </c>
+      <c r="E61" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" ht="13.5">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>neonatal_bulging_fontanel</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Bulging anterior fontanel</t>
+        </is>
+      </c>
+      <c r="E62" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" ht="13.5">
+      <c r="A63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>neonatal_abdominal_distension</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Abdominal distension</t>
+        </is>
+      </c>
+      <c r="E63" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" ht="13.5">
+      <c r="A64" t="s">
+        <v>12</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>neonatal_no_urine</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Not passing urine for a day</t>
+        </is>
+      </c>
+      <c r="E64" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" ht="13.5">
+      <c r="A65" t="s">
+        <v>12</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>neonatal_no_stool</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Not passing stool for a day</t>
+        </is>
+      </c>
+      <c r="E65" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" ht="13.5">
+      <c r="A66" t="s">
+        <v>10</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>has_secondary_neonatal_danger_sign_flag</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>if(selected(${neonatal_not_crying},'yes') or selected(${neonatal_blue_color},'yes') or selected(${neonatal_eye_discharge},'yes') or selected(${neonatal_skin_rash},'yes') or selected(${neonatal_congenital},'yes') or selected(${neonatal_vomiting},'yes') or selected(${neonatal_bulging_fontanel},'yes') or selected(${neonatal_abdominal_distension},'yes') or selected(${neonatal_no_urine},'yes') or selected(${neonatal_no_stool},'yes'),1,0) </t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="1:17" ht="13.5">
+      <c r="A67" t="s">
+        <v>13</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>has_secondary_neonatal_danger_sign_note</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>A danger sign has been identified. Advise the mother to go to any nearby health facility within the next 24 hours so a doctor can look at the baby and help.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>${has_secondary_neonatal_danger_sign_flag}=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:17" ht="13.5">
+      <c r="A68" t="s">
+        <v>13</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>no_secondary_neonatal_danger_sign_note</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>No danger signs were identified in your baby, but if the baby develops any of the signs we discussed, you should go the health facility immediately.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>${has_secondary_neonatal_danger_sign_flag}=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:17" ht="13.5">
+      <c r="A69" t="s">
+        <v>8</v>
+      </c>
+      <c r="B69" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" ht="13.5">
+      <c r="A70" t="s">
+        <v>4</v>
+      </c>
+      <c r="B70" t="s">
+        <v>21</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>(decimal-date-time(today())-decimal-date-time(${child_date_of_birth})) &gt; 42 and (${previous_child_consent}="yes" or selected(${child_consent_today},"yes"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:17" ht="13.5">
+      <c r="A71" t="s">
+        <v>12</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>child_drink</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ASK: Is the child able to drink or breastfeed?</t>
+        </is>
+      </c>
+      <c r="E71" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" ht="13.5">
+      <c r="A72" t="s">
+        <v>12</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>child_vomit</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ASK: Does the child vomit everything?</t>
+        </is>
+      </c>
+      <c r="E72" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" ht="13.5">
+      <c r="A73" t="s">
+        <v>12</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>child_convulsions</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ASK: Has the child recently had any convulsions?</t>
+        </is>
+      </c>
+      <c r="E73" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" ht="13.5">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>child_lethargic</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ASK: Is the child lethargic or unconscious?</t>
+        </is>
+      </c>
+      <c r="E74" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" ht="13.5">
+      <c r="A75" t="s">
+        <v>10</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>refer_child_danger_sign_flag</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>if(selected(${child_drink},"no") or selected(${child_vomit},"yes") or selected(${child_convulsions},"yes") or selected(${child_lethargic},"yes"),1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" spans="1:17" ht="13.5">
+      <c r="A76" t="s">
+        <v>13</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>child_danger_sign_note</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>The child has a danger sign. Advise the mother to go to any nearby health facility within the next 24 hours so a doctor can look at the child and help.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>${refer_child_danger_sign_flag}=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="1:17" ht="13.5">
+      <c r="A77" t="s">
+        <v>13</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>no_child_danger_sign_note</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SAY: No danger signs were identified in your child, but if the child develops any of the signs we discussed, you should go the health facility immediately.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>${refer_child_danger_sign_flag}=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:17" ht="13.5">
+      <c r="A78" t="s">
+        <v>8</v>
+      </c>
+      <c r="B78" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" ht="13.5"/>
+    <row r="108" spans="1:17" ht="13.5"/>
+    <row r="109" spans="1:17" ht="13.5"/>
+    <row r="110" spans="1:17" ht="13.5"/>
+    <row r="111" spans="1:17" ht="13.5"/>
+    <row r="112" spans="1:17" ht="13.5"/>
+    <row r="113" spans="1:17" ht="13.5"/>
+    <row r="114" spans="1:17" ht="13.5"/>
+    <row r="115" spans="1:17" ht="13.5"/>
+    <row r="116" spans="1:17" ht="13.5"/>
+    <row r="117" spans="1:17" ht="13.5"/>
+    <row r="118" spans="1:17" ht="13.5"/>
+    <row r="119" spans="1:17" ht="13.5"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
   <printOptions/>
@@ -1071,216 +1721,20 @@
         </is>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="13.5">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>not_able_feed</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Not able to feed since birth, or stopped feeding well </t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="13.5">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>had_convulsions</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Had convulsions</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="13.5">
-      <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>difficulty_fast_breathing</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Difficulty or fast breathing (Two counts of 60 breaths or more in one minute)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="13.5">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>fever</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Fever or high temperature </t>
-        </is>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="13.5">
-      <c r="A14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>cold</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cold or low temperature </t>
-        </is>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="13.5">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>yellow_pale_palms</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Yellow or pale palms and soles (hands and feet), and lips. Soles should be red/pink.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="13.5">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>no_movement</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Movement only when stimulated, or no movement even on stimulation </t>
-        </is>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="13.5">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>cord_bleeding</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Cord red, bleeding, or draining pus</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="13.5">
-      <c r="A18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>diarrhea</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Diarrhea</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="13.5">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>eyes_pus</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Eyes draining pus</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="13.5">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>skin_boils</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Skin boils</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="13.5">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>excessive_vomiting</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Excessive vomiting</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="13.5">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>excessive_crying</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Excessive crying or restlessness for more than one hour, non-stop</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="13.5">
-      <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>None of the above</t>
-        </is>
-      </c>
-    </row>
+    <row r="10" spans="1:4" ht="13.5"/>
+    <row r="11" spans="1:4" ht="13.5"/>
+    <row r="12" spans="1:4" ht="13.5"/>
+    <row r="13" spans="1:4" ht="13.5"/>
+    <row r="14" spans="1:4" ht="13.5"/>
+    <row r="15" spans="1:4" ht="13.5"/>
+    <row r="16" spans="1:4" ht="13.5"/>
+    <row r="17" spans="1:4" ht="13.5"/>
+    <row r="18" spans="1:4" ht="13.5"/>
+    <row r="19" spans="1:4" ht="13.5"/>
+    <row r="20" spans="1:4" ht="13.5"/>
+    <row r="21" spans="1:4" ht="13.5"/>
+    <row r="22" spans="1:4" ht="13.5"/>
+    <row r="23" spans="1:4" ht="13.5"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
   <printOptions/>

</xml_diff>